<commit_message>
It had forgotten to chech the type
</commit_message>
<xml_diff>
--- a/data/result/error_report.xlsx
+++ b/data/result/error_report.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -450,7 +450,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>93</v>
+        <v>2</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -459,7 +459,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>inv-91</t>
+          <t>inv-0</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -472,23 +472,27 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Original row flagged: Conflict with row 447</t>
+          <t>Original row flagged: Conflict with row 3</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>102</v>
+        <v>3</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>customer_code</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
+          <t>invoice_number</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>INV-0</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>MISSING_REQUIRED</t>
+          <t>COMPOSITE_DUPLICATE</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -496,27 +500,27 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Mandatory field is empty</t>
+          <t>Duplicate of row 2</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>402</v>
+        <v>94</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>customer_code</t>
+          <t>invoice_number</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>CUST-X</t>
+          <t>inv-91</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>PATTERN_MISMATCH</t>
+          <t>COMPOSITE_DUPLICATE</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -524,27 +528,23 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Invalid pattern: CUST-X</t>
+          <t>Original row flagged: Conflict with row 448</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>403</v>
+        <v>103</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
           <t>customer_code</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>CUST-X</t>
-        </is>
-      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>PATTERN_MISMATCH</t>
+          <t>MISSING_REQUIRED</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -552,27 +552,27 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Invalid pattern: CUST-X</t>
+          <t>Mandatory field is empty</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>447</v>
+        <v>403</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>invoice_number</t>
+          <t>customer_code</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>INV-91</t>
+          <t>CUST-X</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>COMPOSITE_DUPLICATE</t>
+          <t>PATTERN_MISMATCH</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -580,13 +580,13 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Duplicate of row 93</t>
+          <t>Invalid pattern: CUST-X</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>503</v>
+        <v>404</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -595,7 +595,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>CUST-Y</t>
+          <t>CUST-X</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -608,27 +608,27 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Invalid pattern: CUST-Y</t>
+          <t>Invalid pattern: CUST-X</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>504</v>
+        <v>448</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>customer_code</t>
+          <t>invoice_number</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>CUST-Y</t>
+          <t>INV-91</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>PATTERN_MISMATCH</t>
+          <t>COMPOSITE_DUPLICATE</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -636,13 +636,13 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Invalid pattern: CUST-Y</t>
+          <t>Duplicate of row 94</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -670,77 +670,77 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>30</v>
+        <v>505</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>customer_code</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>CompanyCompanyCompanyCompanyCompanyCompanyCompanyCompanyCompanyCompanyCompanyCompanyCompanyCompanyCompanyCompanyCompanyCompany 28</t>
+          <t>CUST-Y</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>BUSINESS_RULE_VIOLATION</t>
+          <t>PATTERN_MISMATCH</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Too long (Max: 50)</t>
+          <t>Invalid pattern: CUST-Y</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>302</v>
+        <v>506</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>amount</t>
+          <t>customer_code</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>5000</t>
+          <t>CUST-Y</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>BUSINESS_RULE_VIOLATION</t>
+          <t>PATTERN_MISMATCH</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Constraint: Since status is suspend, this must be None</t>
+          <t>Invalid pattern: CUST-Y</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>703</v>
+        <v>31</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>name</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>invalid_email.com</t>
+          <t>CompanyCompanyCompanyCompanyCompanyCompanyCompanyCompanyCompanyCompanyCompanyCompanyCompanyCompanyCompanyCompanyCompanyCompany 28</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>PATTERN_MISMATCH</t>
+          <t>BUSINESS_RULE_VIOLATION</t>
         </is>
       </c>
       <c r="E12" t="n">
@@ -748,33 +748,169 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Invalid email format</t>
+          <t>Too long (Max: 50)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>202</v>
+        <v>303</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
+          <t>amount</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>5000</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>BUSINESS_RULE_VIOLATION</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>2</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Constraint: Since status is suspend, this must be None</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>704</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>invalid_email.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>PATTERN_MISMATCH</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>2</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Invalid email format: 'invalid_email.com'</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>804</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>amount</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>TEXT_DATA</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>TYPE_MISMATCH</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>2</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Expected float but got: 'TEXT_DATA'</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>75004</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>amount</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>df</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>TYPE_MISMATCH</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Expected float but got: 'df'</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>75005</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>amount</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>MISSING_REQUIRED</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>2</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Mandatory field is empty</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>203</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
           <t>project_code</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>WRONG-CODE</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>PATTERN_MISMATCH</t>
         </is>
       </c>
-      <c r="E13" t="n">
+      <c r="E18" t="n">
         <v>3</v>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>Invalid pattern: WRONG-CODE</t>
         </is>

</xml_diff>